<commit_message>
Update CSR test data and enhance extraction logic
- Modified CSR audio URLs and call IDs in run_csr_test.py to reflect the latest batch from March 13, 2026.
- Improved data extraction logic by updating scope-related fields to pull from the qualification data instead of a removed scope variable.
- Added a new test file, test_scenario_calls.py, to validate unique call scenarios fetched from the Otto API, ensuring no duplicates and at least five scenarios are matched.
</commit_message>
<xml_diff>
--- a/reports/audio_url_test_results_final.xlsx
+++ b/reports/audio_url_test_results_final.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA11"/>
+  <dimension ref="A1:CA21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -3521,6 +3521,2554 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/bd24a254-fe4e-48ef-9c3e-3c3f3adfd68c/4082148782.mp3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nita</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tim</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Roof shingle replacement estimate/quote</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Oh goodness. Hmm. Okay. Okay. Well, I'll have to think about that one because I, yeah, that's, that's, I don't want to pay that. I already paid a, I already paid an inspector to come check the place out, but. | Oh, you don't, it's not a free estimate?</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>new_inquiry</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>customer_rep: Hi, this is Nita from Arizona. We'll first, how can I help?
+home_owner: Oh, hi there. Um, my name is Tim, and I'm over in Palm Creek, resort. And I'm in the, I'm in the process of possibly purchasing a, uh, little park model, but I think the shingles need doing on it. So, um, are you guys in the area, are you?
+customer_rep: Yes, we do service the area, but since you are still in the process on purchasing the, um, property, that we do have a service, um, fee, I mean, we have a fee for the quotation, which is $299. We do have a service, um, fee, I mean, we have a fee for the quotation, which is $299.
+home_owner: Oh, you don't, it's not a free estimate?
+customer_rep: Uh, for the free estimate, uh, we offer free estimate if you already are the owner of the property, but if the property is still in listing, you're, you're selling it, you're the buyer, uh, we're charging for quotation.
+home_owner: oh i see i see is that the way most guys work it?
+customer_rep: Yes, mostly.
+home_owner: Okay, okay. And what, what did you say it would cost?
+customer_rep: Uh two hundred ninety-nine.
+home_owner: Oh goodness. Hmm. Okay. Okay. Well, I'll have to think about that one because I, yeah, that's, that's, I don't want to pay that. I already paid a, I already paid an inspector to come check the place out, but.
+customer_rep: All right.
+home_owner: He suggested that we get a roofer to get a good estimate or a good estimate on, uh, I'd like an estimate even to know what it's gonna cost me to, uh, replace the single phone. Mm-hmm. So… um if ever. Good.
+customer_rep: If that is the case, you can ask the owner of the property if they can, you know, add it to a gift for the, um, house.
+home_owner: Okay, yeah, that might work, great, okay. Thank you.
+customer_rep: Okay, sounds good, sounds good,
+home_owner: I will, uh… All is good. I'll talk to them and see what we can come up with.
+customer_rep: Not a problem. Thank you very much as well. Be safe. Bye-bye.</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>scenario_test_1_88148c4c</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Palm Creek Resort</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="AG12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>Oh goodness, I don't want to pay that, I already paid a, I already paid an inspector to come check the place out, two hundred ninety-nine, it's not a free estimate?</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>unqualified</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>After the caller explained they were considering purchasing a park model and suspected the shingles needed replacement, the rep moved directly to stating there is a $299 quotation fee without first gathering basic details (roof issue, urgency, property address, access, or what the customer needs the estimate for)., When the caller objected to the $299 fee (“Oh goodness... I don't want to pay that”), the rep responded briefly (“All right.”) and did not explore the objection, offer options, or attempt to preserve the lead with a next step., The rep did not complete identification and contact verification (did not confirm the caller’s name, phone number, email, or the exact property address) and did not set a follow-up action before ending the call., The rep did not set expectations about what the paid quotation includes (inspection scope, deliverables, time on site, whether it’s credited toward work, or how it helps with a purchase decision).</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>Confirmed service area availability for the caller’s location., Clearly disclosed the quote/inspection fee amount and the condition for a free estimate (must be the owner)., Maintained a polite, calm tone and closed courteously.</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , </t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="AX12" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>Tim (prospective buyer)</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>Tim is considering purchasing a park model at Palm Creek resort and wants an estimate to replace shingles. He declined the $299 quotation fee because he doesn't want to pay it and plans to talk to the property owner about covering/adding the fee.</t>
+        </is>
+      </c>
+      <c r="BG12" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>Caller (Tim) is considering purchasing a park model in Palm Creek Resort and thinks the shingles need to be redone/replaced., Rep stated the company services the area but charges a $299 quotation fee when the caller is not yet the owner and the property is still in listing; free estimates are for current owners., Tim did not schedule anything on the call and said he will talk to the current owner about possibly covering/including the quotation fee.</t>
+        </is>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>Customer will speak with the current property owner about covering or including the $299 quotation fee., Customer may call back to proceed with a paid quotation or wait until ownership to request a free estimate.</t>
+        </is>
+      </c>
+      <c r="BJ12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>Confirmed service area availability for the caller’s location., Clearly disclosed the quote/inspection fee amount and the condition for a free estimate (must be the owner)., Maintained a polite, calm tone and closed courteously.</t>
+        </is>
+      </c>
+      <c r="BM12" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO12" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP12" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ12" t="inlineStr">
+        <is>
+          <t>Caller is a prospective buyer requesting a roofing estimate/quote for a property they may purchase and discussing the estimate fee—this is a new lead inquiry with pre-sale objection.</t>
+        </is>
+      </c>
+      <c r="BR12" t="inlineStr">
+        <is>
+          <t>New lead asking if company services the area, Requesting an estimate/quote for shingle replacement, Pre-sale objection to $299 quotation fee</t>
+        </is>
+      </c>
+      <c r="BS12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="BT12" t="inlineStr">
+        <is>
+          <t>Palm Creek resort</t>
+        </is>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>Greeting</t>
+        </is>
+      </c>
+      <c r="BW12" t="inlineStr">
+        <is>
+          <t>Identification, Needs Discovery, Qualifying (BANT), Scheduling, Setting Expectations, Close &amp; Confirmation, Objection Handling</t>
+        </is>
+      </c>
+      <c r="BX12" t="n">
+        <v>8</v>
+      </c>
+      <c r="BY12" t="inlineStr">
+        <is>
+          <t>Tim called from Palm Creek Resort because he is in the process of possibly purchasing a small park model and believes the shingles need to be replaced; he wanted an estimate to understand the replacement cost. Nita confirmed the company services the area but explained that estimates are only free for current property owners, and that a $299 quotation fee applies when the property is still listed and the caller is the buyer. Tim expressed concern about paying the fee since he already paid an inspector, and the call ended with Nita suggesting he ask the current owner to cover or include the fee, with Tim saying he would talk to them and see what they can do.</t>
+        </is>
+      </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>I'm in the process of possibly purchasing a, uh, little park model</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/00273c23-da2c-4e1b-b49c-4ff85d4a766a/4082112377.mp3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Nika</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Chase Eatman</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Roof repair (replace/repair fallen roof tiles; no active leak)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Okay. I'm going to need something sooner, so I'll have to call someone else.</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>new_inquiry</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>customer_rep: Hi, this is Nika from Arizona. Of course, how can I help?
+home_owner: Hello, I just needed to. Ooh. see when I can get someone out if possible. I have a repair that needs to be done on a roof. Some tiles had fell- fallen down.
+customer_rep: Oh, okay. Um, is it for a repair? and yeah. Okay. Um, is it leaking inside now?
+home_owner: Say it again.
+customer_rep: is it is it also leaking at your property?
+home_owner: no, there's no leaking.
+customer_rep: Okay, got it. And, um, may I know how old is your roof?
+home_owner: um it's a little over ten years.
+customer_rep: Okay, got it, thank you very much and can you provide me the address?
+home_owner: It's 15227 West Bloomfield Road besides Arizona. by barizona. eight, five, three, seven, nine.
+customer_rep: I'm sorry, A5? three, seven, nine.
+home_owner: Okay, thank you.
+customer_rep: Let me repeat that, uh, one, five, two, two, seven, West. Is it Bokaraton Road? Surprise?
+home_owner: It's Bloomfield, B-L-O-O-M-F-I-E-L-D.
+customer_rep: I'm sorry, B. L. . I.B.L. Bloomfield.
+home_owner: Bloomfield. yeah, bloomfield.
+customer_rep: Okay, got it. Thank you. I got it here now for some minutes. Let me repeat that just to make sure I have the correct information. 15227 West Bloomfield Road in Surprise 85379. that's correct. Okay, and it is more than 10 years. Okay, and it's a tell, and, um, how many stories do you have?
+home_owner: Two.
+customer_rep: Okay, thank you. And are you the owner of the property? Okay, can I have your first name?
+home_owner: Chase?
+customer_rep: Okay. And your last name?
+home_owner: Eatman, E-A-T-M-O-N.
+customer_rep: I'm sorry, can you repeat that?
+home_owner: E. A. T. M. O. N. .
+customer_rep: Okay, thank you very much. And the best phone number that we can reach out 602 is 323856.
+home_owner: Yes.
+customer_rep: And, um, is your property in our HOA?
+home_owner: Yeah.
+customer_rep: okay and lastly can i have ah we have any solar panel.
+home_owner: no.
+customer_rep: No solar, okay. And last you can have your email.
+home_owner: yeah, it's c, the first letter of my name, and then my last name, eatman, e-a-t-m-o-n. A.T.M. away. and then hunter h u n t e r at gmail dot com.
+customer_rep: Thank you. Let me repeat that. Um, your C, first name and then eat mom and hunter at gmail.com.
+home_owner: Yes.
+customer_rep: Okay, thank you. Finally in the line, I'll go ahead and double check our schedule, okay?
+home_owner: Okay. How did you release the book? Okay. If you think if this was the work you got it on the Alright,
+customer_rep: as for tracking here, we do have an availability, uh, next week. We have an availability on Tuesday, uh, 7.30 a.m. to 9 a.m. and then we also have 10 a.m. till 12 p.m., 1 p.m. to 3 p.m. and 4 p.m. till 6 p.m.
+home_owner: Okay. I'm going to need something sooner, so I'll have to call someone else.
+customer_rep: Oh, I see. All right. But if ever that, um, you don't have someone who can, um, assist you before that date, then just let us know, okay?
+home_owner: Okay.
+customer_rep: Yeah, we do apologize. This is the soonest schedule I can offer. Thank you.
+home_owner: Thank you.</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>scenario_test_2_2e229983</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Surprise</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>15227 West Bloomfield Road</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>85379</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="AG13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>in-person</t>
+        </is>
+      </c>
+      <c r="AM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>qualified_but_unbooked</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>The rep opened with a greeting but did not state the company name and did not clearly confirm the caller’s name until later, which weakened identification and professionalism at the start., After learning tiles fell and there was no active leak, the rep did not ask key needs-discovery questions like when it happened, how many tiles, any visible damage, or whether anyone has inspected it, then moved quickly into data collection., Qualifying was incomplete: the rep asked “are you the owner” but did not capture/confirm the homeowner’s response, and did not ask timeline/urgency, other quotes, or any budget/financing considerations., When the customer objected that they needed something sooner, the rep did not attempt to save the appointment by offering alternatives (waitlist/cancellation list, different crew/branch, emergency temporary repair, or checking nearby availability) and instead accepted the loss., The rep did not set expectations for the appointment (what happens during inspection, how long it takes, what the customer receives) and did not complete a close/confirmation (no recap, no confirmation message, no next steps).</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>Asked key diagnostic questions (leak status, roof age, stories) to understand basic situation, Collected and verified critical contact details (address, phone, email) with read-back, Provided multiple appointment windows for the available day</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , , </t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="AX13" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>Chase Eatman (homeowner)</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>Customer requested roof tile repair ("Some tiles had fell- fallen down"), no leaking reported, roof is a little over ten years old, two-story home, HOA, no solar. Offered next-week Tuesday time windows but customer said they need something sooner and will call someone else; follow up if earlier availability opens.</t>
+        </is>
+      </c>
+      <c r="BG13" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>Customer needs a roof repair because some tiles have fallen down; customer stated there is no leaking inside., Property details collected: tile roof, a little over 10 years old, two-story home, in an HOA, no solar panels; address provided as 15227 West Bloomfield Road, Surprise, AZ 85379., Scheduling outcome: soonest availability offered was next week Tuesday with multiple time windows; customer declined due to needing sooner service and said they would call someone else.</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>Customer to contact another roofing company for a sooner appointment., If the customer cannot find earlier service, customer may call back to schedule one of the offered Tuesday time windows next week.</t>
+        </is>
+      </c>
+      <c r="BJ13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>Asked key diagnostic questions (leak status, roof age, stories) to understand basic situation, Collected and verified critical contact details (address, phone, email) with read-back, Provided multiple appointment windows for the available day</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP13" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ13" t="inlineStr">
+        <is>
+          <t>Caller is a homeowner requesting a roof repair and trying to schedule the soonest available appointment; this is a new service inquiry/appointment-setting interaction even though they ultimately decline due to timing.</t>
+        </is>
+      </c>
+      <c r="BR13" t="inlineStr">
+        <is>
+          <t>new repair/service request, attempt to schedule an appointment/inspection window, no indication of existing contract or ongoing job status</t>
+        </is>
+      </c>
+      <c r="BS13" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>15227 West Bloomfield Road, Surprise, Arizona 85379</t>
+        </is>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Needs Discovery, Scheduling (attempted)</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>Qualifying (BANT), Setting Expectations, Objection Handling, Close &amp; Confirmation</t>
+        </is>
+      </c>
+      <c r="BX13" t="n">
+        <v>7</v>
+      </c>
+      <c r="BY13" t="inlineStr">
+        <is>
+          <t>Chase Eatman called to request a roof repair because some roof tiles had fallen down, but confirmed there is currently no interior leaking. The representative gathered property and contact details, including that the roof is a tile roof a little over 10 years old, the home is two stories, it is in an HOA, and there are no solar panels. The rep offered the soonest available appointment windows for next week on Tuesday (7:30–9:00 AM, 10:00 AM–12:00 PM, 1:00–3:00 PM, or 4:00–6:00 PM). The customer said they needed something sooner and would call someone else, and the rep advised them to call back if they could not find earlier help elsewhere.</t>
+        </is>
+      </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>I'm going to need something sooner, so I'll have to call someone else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/c0183543-60e4-434f-a247-89ec9ef8e1e3/4081871096.mp3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Bronte</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Roof tile repair/replacement (replace missing roof tiles; quote requested)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>service_not_offered</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>quote_only</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>customer_rep: Thank you for calling Arizona Rebirth. This is Bronte. How can I help you?
+home_owner: hi, i was wondering if i get a, a, a quote on, um, repair of some roof tiles that i have missing?
+customer_rep: Um, yeah, how old is the roof?
+home_owner: I'm not sure.
+customer_rep: okay um are you the property owner?
+home_owner: yes, i am the copy of it.
+customer_rep: Okay, um, when did you purchase the house?
+home_owner: ah about five years ago.
+customer_rep: Okay. And are you experiencing like any issues with the roof or you're just wanting the tiles replaced?
+home_owner: Yeah, I just need the tiles replaced. Um, I got a message from H-O-8 saying that there's some missing tiles, and so I just wanted to get a quote and see how much it would be to replace them.
+customer_rep: Okay, yeah. Um, fortunately it does sound like a smaller repair, but right now those kinds of jobs are just a little bit out of our scope. We do work with a, um, different roofing company, their name is XRP, and they specialize in like smaller jobs and repairs, so I can give you their phone number if you wanted to give them a call.
+home_owner: It's called XRP. Okay, I'll, I'll look them up and give them a call. Thank you.
+customer_rep: Yeah, have a good one.
+home_owner: Thank you very much.</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>scenario_test_3_cc5d0fb9</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="AG14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>I just wanted to get a quote and see how much it would be to replace them</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>qualified_service_not_offered</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>After the customer asked for a quote on missing roof tiles, the rep quickly concluded the job was out of scope and referred the caller to another company without explaining pricing limitations or the need for an in-person assessment to provide an accurate quote., The rep did not attempt to schedule an appointment or explore whether the situation could qualify for their services (e.g., inspection to confirm if there is underlying damage) before ending the call., The rep did not collect or verify the caller’s contact information (name, phone, address/email) at any point, even to support a referral or future follow-up., The close was abrupt and did not confirm the customer successfully received the referral information or offer to send it via text/email.</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>Opened with a professional greeting including company name and rep name., Asked basic qualifying questions (roof age, ownership, purchase timing) and clarified whether there were active issues vs. simple replacement.</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , </t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="AX14" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>Homeowner (property owner)</t>
+        </is>
+      </c>
+      <c r="BG14" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH14" t="inlineStr">
+        <is>
+          <t>Homeowner requested a quote to repair/replace missing roof tiles., Caller confirmed they are the property owner and purchased the house about five years ago; they were unsure of the roof’s age., Arizona Rebirth stated small repair jobs are out of scope and referred the homeowner to a partner company named XRP for the repair.</t>
+        </is>
+      </c>
+      <c r="BI14" t="inlineStr">
+        <is>
+          <t>Homeowner to look up and contact XRP for a quote on replacing the missing roof tiles., No appointment scheduled with Arizona Rebirth due to the job being out of scope.</t>
+        </is>
+      </c>
+      <c r="BJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t>Opened with a professional greeting including company name and rep name., Asked basic qualifying questions (roof age, ownership, purchase timing) and clarified whether there were active issues vs. simple replacement.</t>
+        </is>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO14" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP14" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ14" t="inlineStr">
+        <is>
+          <t>Caller is a property owner requesting a quote to replace missing roof tiles, which is a new lead inquiry even though the company ultimately refers the job out as out of their scope.</t>
+        </is>
+      </c>
+      <c r="BR14" t="inlineStr">
+        <is>
+          <t>new lead requesting a quote/estimate, service need described (missing roof tiles repair)</t>
+        </is>
+      </c>
+      <c r="BS14" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="BU14" t="inlineStr">
+        <is>
+          <t>Small roof tile repair jobs are out of scope for Arizona Rebirth; referred to another roofing company (XRP).</t>
+        </is>
+      </c>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Understand the Need</t>
+        </is>
+      </c>
+      <c r="BW14" t="inlineStr">
+        <is>
+          <t>Educate on need for in-person assessment, Handle objections about inspection, Attempt to schedule (if appropriate), Close</t>
+        </is>
+      </c>
+      <c r="BX14" t="n">
+        <v>6</v>
+      </c>
+      <c r="BY14" t="inlineStr">
+        <is>
+          <t>The homeowner called Arizona Rebirth to request a quote to repair/replace some missing roof tiles. The representative asked about the roof’s age (the homeowner was unsure), confirmed the caller is the property owner, and learned the home was purchased about five years ago. The homeowner said they were not experiencing other issues and only needed tiles replaced after receiving a message from “H-O-8” noting missing tiles. The representative explained that small tile repair jobs are currently out of Arizona Rebirth’s scope and referred the homeowner to a partner company, XRP, that specializes in smaller repairs; the homeowner agreed to look them up and call, and the call ended without an appointment being scheduled.</t>
+        </is>
+      </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>I got a message from H-O-8 saying that there's some missing tiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/eb359c0a-02e2-4e94-b018-b3585c8a4024/4081765241.mp3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Diva</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Commercial roof repair (hole/leak) inspection/estimate</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>new_inquiry</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>customer_rep: Thank you for calling Arizona Roofers. My name is Diva. How can I help you?
+home_owner: Hi, I have received a call from you guys about an inquiry that I've had for a roof repair in Sedona. And I got cut off with you because I was going into an appointment yesterday. But I wanted to finish that call and schedule a time.
+customer_rep: No worries. It looks like it was my colleague Grante.
+customer_rep: Yeah. So this is a commercial building?
+home_owner: Yeah.
+customer_rep: I'm trying to read what she has. Do you know how old the commercial building is?
+home_owner: I do not.
+customer_rep: Okay, is this a single story?
+home_owner: Okay, one moment, please.
+customer_rep: Do you know how much square footage it is?
+home_owner: So that's a hard question because there's two roofs. It's a building that's like split in the middle and we only need the right side. What's that?
+customer_rep: Okay, no worries. I did get.
+home_owner: Oh, actually the people that we had bond with before but were trying to switch just because they had the warranty, but they didn't abide by it. Now I miss to pay for a hole in the roof. So we're trying to switch to somebody else. They did send me a. And it might be on there.
+customer_rep: Okay. It's okay. If you don't have it now, you can let your technician know then and there. So are you the property owner then?
+home_owner: Yes.
+customer_rep: Did you want me to add in an email to your contact info? We usually send the proposal to this.
+home_owner: Yes.
+customer_rep: Okay, I'm ready.
+home_owner: The roof side is 21 squares. Okay. I don't know what that means. Is that what you needed?
+customer_rep: Well, I could. I'll note that down. Okay. And then an email.
+home_owner: R waters. R w a t t e r s at c as in cat. A as in apple. C as in paul. Servicing.com.
+customer_rep: Perfect. All right, so for commercial jobs, we have our technician actually give you a call and schedule a time that works best for both of you. Okay. We only have a few technicians are able to handle them, so. Yeah, I have all your information down. I'll go ahead and tag that technician and he'll be reaching out to you shortly.
+home_owner: Okay, perfect. Thank you so much. Have a good night.
+customer_rep: No problem. You too. Bye.
+home_owner: Bye.</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>scenario_test_4_334fff68</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Commercial technician to call the customer to schedule an on-site appointment for the Sedona commercial roof repair.</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Sedona</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="AG15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>Now I miss to pay for a hole in the roof.</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>unqualified</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>After the customer said they wanted to "finish that call and schedule a time," the rep did not book an appointment or even provide a specific callback window; instead, she ended with "he'll be reaching out to you shortly" without locking a date/time or SLA., The rep asked building age/stories/square footage but never clarified the actual repair need (e.g., leak location, type of damage, urgency, active water intrusion) before moving to the handoff., When the customer explained they are switching because the prior company “had the warranty, but they didn't abide by it,” the rep acknowledged but did not probe or reassure how Arizona Roofers handles warranties/service commitments., The rep did not set expectations for the next step (what the technician will do, approximate appointment length, what the customer should have ready, and how/when proposals are delivered).</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>Used a professional greeting with company name and rep name., Confirmed decision-maker status by asking if the caller is the property owner., Collected email for proposal delivery and reassured customer they can provide missing details to the technician.</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , </t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="AX15" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>Property owner (caller)</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>Commercial roof repair in Sedona. Building has two roofs; only the right side needs work. Customer estimates roof side is '21 squares'. Prior contractor had a warranty but 'they didn't abide by it'; customer wants to switch providers. Email provided: rwaters@cacpaulservicing.com. Commercial technician needs to call customer to schedule.</t>
+        </is>
+      </c>
+      <c r="BG15" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>Customer requested roof repair for a commercial building in Sedona and called back to finish scheduling after being cut off the previous day., Property details provided: commercial building with two roof sections; only the right side needs work; roof side noted as 21 squares; building age unknown., Customer is switching from a previous contractor due to a warranty not being honored and mentioned needing to pay for a hole in the roof; rep collected email (rwaters@cacpservicing.com) and advised a commercial technician will call to schedule.</t>
+        </is>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>Assigned commercial technician contacts the homeowner shortly to coordinate a date/time for the visit., During the visit/call, technician confirms missing details (building age, story count, square footage and scope for the right-side roof) and prepares a proposal to send via email.</t>
+        </is>
+      </c>
+      <c r="BJ15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>Used a professional greeting with company name and rep name., Confirmed decision-maker status by asking if the caller is the property owner., Collected email for proposal delivery and reassured customer they can provide missing details to the technician.</t>
+        </is>
+      </c>
+      <c r="BM15" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO15" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP15" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ15" t="inlineStr">
+        <is>
+          <t>Caller is a property owner requesting roof repair for a commercial building and is calling back to schedule an inspection/appointment; contact details are collected and a technician will call to set a time.</t>
+        </is>
+      </c>
+      <c r="BR15" t="inlineStr">
+        <is>
+          <t>new lead/inquiry for roof repair, appointment setting for technician/inspection, proposal/estimate process (email for proposal)</t>
+        </is>
+      </c>
+      <c r="BS15" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="BT15" t="inlineStr">
+        <is>
+          <t>Sedona</t>
+        </is>
+      </c>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Needs Discovery, Qualifying (BANT), Close &amp; Confirmation</t>
+        </is>
+      </c>
+      <c r="BW15" t="inlineStr">
+        <is>
+          <t>Scheduling (if applicable), Setting Expectations, Objection Handling (if objections arose)</t>
+        </is>
+      </c>
+      <c r="BX15" t="n">
+        <v>7</v>
+      </c>
+      <c r="BY15" t="inlineStr">
+        <is>
+          <t>The homeowner called Arizona Roofers to continue a previously interrupted conversation and schedule service for a roof repair on a commercial building in Sedona. The representative reviewed the prior notes, asked about the building’s age, whether it is single story, and the square footage, but the caller did not know the age and explained the building has two roof sections and they only need work on the right side. The caller shared they are switching contractors because a prior company did not honor a warranty and they now need to pay to address a hole in the roof. The rep collected an email address for sending a proposal and noted the roof area as “21 squares,” then explained that for commercial jobs a qualified technician will call the customer to coordinate a mutually convenient appointment. The call ended with the technician to reach out shortly to schedule.</t>
+        </is>
+      </c>
+      <c r="CA15" t="inlineStr">
+        <is>
+          <t>I wanted to finish that call and schedule a time., I was going into an appointment yesterday.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/4da88a74-f129-481d-92d4-626c5a728835/4081742162.mp3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bronte</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Tiled roof pricing estimate (cost per square)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>send_info</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Provide pricing guidance to the customer for current cost per square of a tiled roof</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>quote_only</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>customer_rep: Thank you for calling Arizona Roofers. This is Bronte. How can I help you?
+home_owner: Yes, hi. This is Adam. I'm wondering, how much is a square of a tiled roof cost now?
+customer_rep: I'm not too sure, to be honest with you. Usually we don't give prices over the phone.
+home_owner: Oh, okay. Thank you very much, then.
+customer_rep: Yeah, I'm a good one.
+home_owner: You too.</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>scenario_test_5_8b5c1e22</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Provide pricing guidance to the customer for current cost per square of a tiled roof</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="AG16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>how much is a square of a tiled roof cost now?</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>qualified_but_unbooked</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>When the homeowner asked, "how much is a square of a tiled roof cost now?", the rep responded that they were not sure and that the company usually doesn't give prices over the phone, without providing any context or next step., After the customer accepted the no-phone-quote response and said, "Oh, okay. Thank you very much, then.", the rep did not attempt to save the call by asking discovery questions or offering to schedule an inspection., The rep ended the call with an unclear/unprofessional closing: "Yeah, I'm a good one."</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Opened with a professional greeting including company name and rep name.</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , </t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="AX16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>Adam (homeowner)</t>
+        </is>
+      </c>
+      <c r="BG16" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>Caller (Adam) asked for the current cost per square for a tiled roof., Rep (Bronte) stated she was not sure and that they usually don’t give prices over the phone., The call ended politely with no appointment, inspection, or follow-up scheduled.</t>
+        </is>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>Customer would need to request an on-site estimate/inspection to receive pricing., If the customer calls back, collect property details and schedule an appointment.</t>
+        </is>
+      </c>
+      <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK16" t="inlineStr">
+        <is>
+          <t>Opened with a professional greeting including company name and rep name.</t>
+        </is>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO16" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP16" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="BQ16" t="inlineStr">
+        <is>
+          <t>Caller is a potential new lead asking about current roofing cost per square; this is a pre-purchase pricing inquiry even though no estimate/appointment was set.</t>
+        </is>
+      </c>
+      <c r="BR16" t="inlineStr">
+        <is>
+          <t>new lead pricing inquiry, decision-making about purchase (cost question)</t>
+        </is>
+      </c>
+      <c r="BS16" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="BV16" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification (partial: company + rep name)</t>
+        </is>
+      </c>
+      <c r="BW16" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification (missing: capture/confirm caller info beyond name), Understand the Need, Educate on need for in-person assessment (WHY), Handle objections about inspection, Attempt to schedule (if appropriate), Close</t>
+        </is>
+      </c>
+      <c r="BX16" t="n">
+        <v>7</v>
+      </c>
+      <c r="BY16" t="inlineStr">
+        <is>
+          <t>Adam called Arizona Roofers to ask how much a square of a tiled roof costs. Bronte explained that she wasn’t sure and that the company usually does not provide pricing over the phone. Adam thanked her and ended the call without scheduling an inspection or estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/c6c4fff3-72d5-42d5-9cb4-16b8272e3d3b/4079556188.mp3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mika</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Roof inspection (escrow/home purchase inspection)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>check_availability</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Check inspection availability for 2026-03-14 and inform the customer of open time slots</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>new_inquiry</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>customer_rep: Hi, this is Mika from Arizona Roofers. How can I help?
+home_owner: Hey, so we just entered into escrow on a house and do you guys do roof inspections?
+customer_rep: Yes, we do. So are you buying or selling the property?
+home_owner: Buying.
+customer_rep: Buying. Okay. Since you still don't own the property, we do inspection, but it will be for 299.
+home_owner: How much?
+customer_rep: 299.
+home_owner: Okay. And then I might let me talk to my realtor really quick on it. But do they have available. Do you know if there's availability tomorrow?
+customer_rep: Let me check our availability. Can you provide me the complete address?
+home_owner: Yeah, just a second.
+customer_rep: Sure.
+home_owner: Okay, are you ready for it?
+customer_rep: Go ahead.
+home_owner: 1664. I'm sorry, 15. 1664. Okay. East Olive Avenue. Okay, that's in Gilbert, Arizona.
+customer_rep: Okay. All right, let me repeat that. 1664 East Olive Avenue, Gilbert, Arizona, 85234.
+home_owner: Yep. Thank you kindly. Send the line. I'll go ahead and double check right now.
+customer_rep: Okay, thank you.
+home_owner: Okay, thank you. Hello?
+customer_rep: Hi. Yes, thank you very much for patiently waiting on the line. As per tracking, we are already fully booked for this week. Next availability that we have, that will be next week, which is Monday.
+home_owner: Okay, let me check and I'll get back to you.
+customer_rep: All right, not a problem. Anyway, thank you very much for your time as well. And have a blessed day to you. Be safe.
+home_owner: You too. Bye.</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>scenario_test_6_c383236d</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Check inspection availability for 2026-03-14 and inform the customer of open time slots</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Gilbert</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>1664 East Olive Avenue</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>1664</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="AG17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>it will be for 299, How much?, 299</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>qualified_but_unbooked</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>After the customer asked for a roof inspection for an escrow purchase, the rep moved quickly to price and scheduling without asking any needs-discovery questions about the roof condition, concerns, or what the inspection is intended to cover., The rep did not collect the caller’s name or any callback number/email, and the call ended with the customer saying they would get back to the company., When the rep found no availability this week, they only offered a single option (“next week, Monday”) and did not attempt to secure a tentative appointment or offer alternatives like other days, time windows, waitlist, or cancellations., The rep did not set expectations for the inspection service (what the $299 includes, how long it takes, what deliverables the customer receives, and payment/authorization process), which left the customer with minimal information to decide., The rep did not perform a clear close and confirmation step—no recap of next steps, no offer to send confirmation, and no plan for follow-up after the customer said they would check and call back.</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>Professional greeting with company name and rep name, Clarified whether customer is buying or selling to determine inspection context and pricing, Confirmed and repeated the full address back to the customer for accuracy, Used polite hold language and thanked the customer for waiting</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , , </t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="AX17" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC17" t="inlineStr">
+        <is>
+          <t>Home owner (buyer), Realtor</t>
+        </is>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>Buyer in escrow requesting a roof inspection for 1664 East Olive Avenue, Gilbert, AZ 85234. Inspection quoted at $299. Customer asked about availability tomorrow but company is fully booked this week; next available is Monday next week. Customer said they will check with their realtor and call back.</t>
+        </is>
+      </c>
+      <c r="BG17" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>Customer requested a roof inspection for a home they are buying and currently in escrow., Rep stated the inspection cost would be $299 because the customer does not yet own the property., Scheduling check showed no availability this week; next availability offered was next Monday (2026-03-16), and the customer said they would get back after checking with their realtor.</t>
+        </is>
+      </c>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>Customer to consult their realtor about proceeding with the $299 inspection., Customer to call back to schedule for the next available slot (Monday, 2026-03-16) if they decide to move forward.</t>
+        </is>
+      </c>
+      <c r="BJ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK17" t="inlineStr">
+        <is>
+          <t>Professional greeting with company name and rep name, Clarified whether customer is buying or selling to determine inspection context and pricing, Confirmed and repeated the full address back to the customer for accuracy, Used polite hold language and thanked the customer for waiting</t>
+        </is>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO17" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP17" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>Caller is a prospective home buyer requesting a paid roof inspection and asking about scheduling availability, indicating a new service inquiry/appointment-setting opportunity.</t>
+        </is>
+      </c>
+      <c r="BR17" t="inlineStr">
+        <is>
+          <t>new lead requesting roof inspection, appointment scheduling/availability discussion, price inquiry for inspection</t>
+        </is>
+      </c>
+      <c r="BS17" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="BT17" t="inlineStr">
+        <is>
+          <t>1664 East Olive Avenue, Gilbert, Arizona 85234</t>
+        </is>
+      </c>
+      <c r="BV17" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Scheduling (partial)</t>
+        </is>
+      </c>
+      <c r="BW17" t="inlineStr">
+        <is>
+          <t>Needs Discovery, Qualifying (BANT), Setting Expectations, Close &amp; Confirmation, Objection Handling (light)</t>
+        </is>
+      </c>
+      <c r="BX17" t="n">
+        <v>7</v>
+      </c>
+      <c r="BY17" t="inlineStr">
+        <is>
+          <t>The caller, who is in escrow and buying a home, asked Arizona Roofers whether they perform roof inspections and inquired about next-day availability. The representative confirmed inspections are available but explained that because the caller does not yet own the property, the inspection fee would be $299. After the caller provided the address (1664 East Olive Avenue, Gilbert, AZ 85234), the representative checked scheduling and reported the company was fully booked for the rest of the week, with the next available appointment on Monday of the following week. The caller said they would check with their realtor and get back to the company, and the call ended without an appointment being scheduled.</t>
+        </is>
+      </c>
+      <c r="CA17" t="inlineStr">
+        <is>
+          <t>we just entered into escrow on a house, availability tomorrow, Next availability that we have, that will be next week, which is Monday</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/ddccb9c0-fce8-4eb5-81bd-5e738cb95979/4078581674.mp3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Travis</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Miranda</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Roof/skylight inspection and estimate for storm damage/issues after recent roof replacement</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>service_not_offered</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>send_details</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Provide customer Miranda with referral contact details for Jonathan at XRP Roofing</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>service_call</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>customer_rep: Thank you for calling Arizona Roofers. My name is Travis. Can I start with your name?
+home_owner: Miranda.
+customer_rep: Hey, Miranda, what's going on? How can we help?
+home_owner: We had a storm damage almost two years ago. And we had a contractor through our middleman, Accuserve, with our USAA come out and do work. And we've had to have our skylights replaced twice now. Accuserve said that we can have our own inspector inspection and estimate given for through who we choose. And I was trying to get that set up.
+customer_rep: Yeah, I could probably come out and take a look. What's the address for you? Let me get you pulled up.
+home_owner: 17128 West Kaya. Carmela, Mariana, Arizona. 85653 West Calle, Arizona.
+customer_rep: Did I hear that right? Calle Carmela. Carmela, that's right. Yeah. 85653.
+home_owner: Yes.
+customer_rep: Gotcha. Let me take a look here. Brenda, how old is the roof?
+home_owner: Less than a. It was changed out last May.
+customer_rep: Man, you guys just put it up there and you're having so many issues with it. I am sorry. That's garbage. We've had terrible control. I'm sorry. That sucks. Has USAA been helping you out at all?
+home_owner: No, it's extra. Not great.
+customer_rep: Okay, let me see here. Let's see. Miranda, I do want to apologize. I was looking at the area and I was trying to see if I can get any technicians out there. Unfortunately, it's not in an area that we would service. But I can refer you to somebody who might be able to help you out. Would you be okay with that?
+home_owner: Yeah, that works.
+customer_rep: Okay. His name is Jonathan. He works with XRP Roofing. Let me know when you're ready.
+home_owner: Okay. All right, I'm ready.
+customer_rep: His phone number is going to be 600-283-3761.
+home_owner: Yeah. Okay.
+customer_rep: Give him a call. See if he can come on out and help you out.
+home_owner: Okay.
+customer_rep: All right. Thank you. Talk to you soon. Bye.
+home_owner: Bye. Bye. Bye.</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>scenario_test_7_b228486b</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Provide customer Miranda with referral contact details for Jonathan at XRP Roofing</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>17128 West Kaya</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>85653</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="AG18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>No, it's extra.</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>unqualified</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>After the customer provided an address that was confusing/inconsistent, the rep moved forward and then concluded the location was out of the service area without fully confirming the complete address (street, city, ZIP) or a callback number/email., When providing the referral, the rep gave only a name and phone number and ended the call without setting expectations (what to say, what services to request, expected response time, or whether Arizona Roofers will follow up)., The rep used negative/unprofessional phrasing while empathizing, which can come across as careless or inflammatory.</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>Opened with company name, rep name, and asked for the caller's name., Allowed the customer to explain the situation and summarized enough to propose a next step., Showed empathy and apologized for the customer's repeated issues., Provided an alternative solution by referring to another roofer when out of service area.</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , </t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="AX18" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AY18" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AZ18" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>Miranda (homeowner)</t>
+        </is>
+      </c>
+      <c r="BG18" t="b">
+        <v>0</v>
+      </c>
+      <c r="BH18" t="inlineStr">
+        <is>
+          <t>Customer (Miranda) requested an inspection and estimate from a contractor of her choice after prior storm-damage work coordinated through Accuserve/USAA and repeated skylight replacements (twice)., Property address provided: 17128 W Calle Carmela, AZ 85653; roof was changed out last May (less than a year old per caller)., Arizona Roofers does not service the customer’s area, so the rep referred her to Jonathan at XRP Roofing (600-283-3761).</t>
+        </is>
+      </c>
+      <c r="BI18" t="inlineStr">
+        <is>
+          <t>Customer to call Jonathan at XRP Roofing (600-283-3761) to request an inspection/estimate., No further steps with Arizona Roofers were scheduled because the address is outside their service area.</t>
+        </is>
+      </c>
+      <c r="BJ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK18" t="inlineStr">
+        <is>
+          <t>Opened with company name, rep name, and asked for the caller's name., Allowed the customer to explain the situation and summarized enough to propose a next step., Showed empathy and apologized for the customer's repeated issues., Provided an alternative solution by referring to another roofer when out of service area.</t>
+        </is>
+      </c>
+      <c r="BM18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO18" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP18" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BQ18" t="inlineStr">
+        <is>
+          <t>Caller requests an independent inspection and estimate for roof/skylight issues; rep attempts to schedule a technician visit (new lead/appointment setting), though they ultimately refer out due to service area.</t>
+        </is>
+      </c>
+      <c r="BR18" t="inlineStr">
+        <is>
+          <t>Requested inspection/estimate through a contractor of their choice, Rep discussed coming out to take a look and asked for address/roof age (lead qualification)</t>
+        </is>
+      </c>
+      <c r="BS18" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BT18" t="inlineStr">
+        <is>
+          <t>17128 West Kaya, Calle Carmela, Mariana, Arizona. 85653</t>
+        </is>
+      </c>
+      <c r="BU18" t="inlineStr">
+        <is>
+          <t>Outside service area</t>
+        </is>
+      </c>
+      <c r="BV18" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Understand the Issue, Empathy &amp; Acknowledgment, Propose Solution/Next Steps, Close</t>
+        </is>
+      </c>
+      <c r="BW18" t="inlineStr">
+        <is>
+          <t>Set Expectations</t>
+        </is>
+      </c>
+      <c r="BX18" t="n">
+        <v>6</v>
+      </c>
+      <c r="BY18" t="inlineStr">
+        <is>
+          <t>Miranda called Arizona Roofers seeking to set up an independent roof inspection and estimate after storm damage from almost two years ago and ongoing issues following work arranged through Accuserve with USAA, including having skylights replaced twice. Travis gathered the property address (17128 W Calle Carmela, AZ 85653) and learned the roof was replaced last May. After checking service availability, Travis explained the location is outside their service area and offered a referral; Miranda agreed, and Travis provided Jonathan at XRP Roofing’s phone number for her to contact.</t>
+        </is>
+      </c>
+      <c r="CA18" t="inlineStr">
+        <is>
+          <t>We had a storm damage almost two years ago., It was changed out last May., we've had to have our skylights replaced twice now</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/add722b1-c29f-4615-b389-4d29773d5958/st_309419607.mp3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Jackie</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Miles</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Porch roof repair/estimate (possible fascia/plywood/boarding replacement under tile due to deterioration)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Okay, Let me call you back once I've consulted someone else, and then we can do that.</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>new_inquiry</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>customer_rep: Good morning and thank you for calling Lions Roofing. My name is Jackie. How may I help you?
+home_owner: Yes, I tried to call you earlier and you didn't answer. So you called me back just a minute ago and I'm returning your call because I missed your call. But I have a residence in South Tempe and the roof of the porch I think needs some possible structural repair. But I don't know that you do that work, do you?
+customer_rep: I'm a little confused on you're asking if we do like re roofs or.
+home_owner: Well, the. The repair is to a porch and it may need some replacement of boarding in order to correct the problem with the deterioration of a board or two in the roof.
+customer_rep: Okay, and you said one of my co workers gave you a call?
+home_owner: Yeah, well, yeah, that's right. I had called earlier and nobody answered. So apparently my number was left behind and so someone called me and I missed the call.
+customer_rep: All right, can I get your name please?
+home_owner: Well, just a minute. The question I have before we go any further is do you do small repairs like that or do you do only roofs, retiling and things of the house roof itself?
+customer_rep: We do repairs, we do re roofs. But you're looking for a repair on a porch roof?
+home_owner: Yeah, As I say, the wood structure underneath the tiles you see may need replacement. Maybe I should talk to a technician first.
+customer_rep: Okay, give me one moment. You say in the wood tile, the wood structure under the tile might need replaced.
+home_owner: Yeah, I'll speak to somebody about that, an estimator. Is there anybody available I could speak to now?
+customer_rep: Actually, give me one moment. Let me reach out to one of my technicians, make sure that we do this and if we do, I can get you on our schedule for our guys to come out and give you that estimate.
+home_owner: Yeah, if he may not do that work. So if I could talk to him now, please.
+customer_rep: All right, give me one moment. Let me place you on a brief hold. But real quick, can I get your name so that I can let my co workers know?
+home_owner: My name is Miles.
+customer_rep: Miles, that's right.
+home_owner: So just go ahead and transfer me if you can.
+customer_rep: Give me one moment. Let me place you on a brief hold. Miles. Okay, It. Hi Miles, are you still with me?
+home_owner: Yeah, I'm right here.
+customer_rep: So sorry for that hold. So I was able to speak with my technician. Unfortunately, I'm not able to pat you through right now. He is at a customers. But we can absolutely get somebody out there to take a look at what's going on and to give you an estimate. Because if it is for like the fascia or plywood that is under the tile. We absolutely get that taken care of for you, but we would have to have a technician come out and see what's going on.
+home_owner: Okay, so in other words, the technician, does he come in a truck so that he has a ladder?
+customer_rep: Yes.
+home_owner: Okay. And is the truck or the van marked as lions?
+customer_rep: Yes, it would say lions roofing, I do believe.
+home_owner: Okay, good. When can someone come by?
+customer_rep: I do have availability tomorrow.
+home_owner: Okay. What time?
+customer_rep: I've got morning or afternoon? I just need some more information to get you on our schedule. I would need to create an account for you.
+home_owner: Okay, Let me call you back once I've consulted someone else, and then we can do that.
+customer_rep: All righty. And thank you very much. Bye bye.
+home_owner: You're very welcome. Bye bye.</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>scenario_test_8_a99fa915</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Tempe</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AG19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>in-person</t>
+        </is>
+      </c>
+      <c r="AM19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>qualified_but_unbooked</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>After the customer described the porch roof structural/wood deterioration, the rep did not ask key diagnostic questions (how long it’s been happening, any active leaks, extent of rot, roof type/material, access constraints) and moved toward scheduling/account creation., The rep did not complete identification/verification details needed to schedule (address, best callback number/email) and only captured the caller’s first name right before placing them on hold., When the customer said they needed to consult someone else and would call back, the rep accepted the brush-off without attempting to save the appointment or set a concrete follow-up plan., The rep did not set expectations for what the technician visit includes (inspection steps, duration, estimate delivery, options, next steps) before offering availability., The rep showed confusion early and did not confidently clarify the service request, which led to repeated back-and-forth before progressing.</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Professional greeting with company name and rep name, Attempted to confirm service capability with a technician before committing, Answered customer questions about technician arrival (ladder/truck and marked vehicle) and offered availability for tomorrow</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, , , , </t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="AX19" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AY19" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AZ19" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>Miles (homeowner)</t>
+        </is>
+      </c>
+      <c r="BF19" t="inlineStr">
+        <is>
+          <t>Miles has a residence in South Tempe and wants a porch roof repair; possible structural wood repair/replacement ("replacement of boarding" / "wood structure underneath the tiles" / fascia or plywood under tile). Rep confirmed they can send a technician with a ladder/marked Lions Roofing truck and had availability tomorrow (morning or afternoon), but customer said: "Let me call you back once I've consulted someone else."</t>
+        </is>
+      </c>
+      <c r="BG19" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH19" t="inlineStr">
+        <is>
+          <t>Customer (Miles) needs a porch roof repair in South Tempe and believes the wood structure/boarding under the tile may be deteriorated and need replacement., Rep confirmed Lions Roofing can likely handle repairs involving fascia/plywood under tile but requires an on-site technician visit to assess and provide an estimate; technician was not available to speak live during the call., Rep offered appointment availability for tomorrow (2026-03-14) morning or afternoon, but the customer declined to book and said he would call back after consulting someone else; customer also asked that the technician arrive with a ladder and in a marked Lions Roofing truck/van.</t>
+        </is>
+      </c>
+      <c r="BI19" t="inlineStr">
+        <is>
+          <t>Customer to call back after consulting someone else to provide details needed to create an account and schedule an on-site estimate., If the customer calls back, schedule a technician visit for the porch roof inspection/estimate (morning or afternoon on 2026-03-14 was offered).</t>
+        </is>
+      </c>
+      <c r="BJ19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK19" t="inlineStr">
+        <is>
+          <t>Professional greeting with company name and rep name, Attempted to confirm service capability with a technician before committing, Answered customer questions about technician arrival (ladder/truck and marked vehicle) and offered availability for tomorrow</t>
+        </is>
+      </c>
+      <c r="BM19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO19" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP19" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BQ19" t="inlineStr">
+        <is>
+          <t>Homeowner is a new lead asking if the company can perform a porch roof structural/wood repair and requests scheduling for a technician to come out and provide an estimate.</t>
+        </is>
+      </c>
+      <c r="BR19" t="inlineStr">
+        <is>
+          <t>new service inquiry/repair request, request to schedule technician visit, request for estimate/inspection availability</t>
+        </is>
+      </c>
+      <c r="BS19" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="BT19" t="inlineStr">
+        <is>
+          <t>South Tempe</t>
+        </is>
+      </c>
+      <c r="BV19" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Needs Discovery, Scheduling (partial)</t>
+        </is>
+      </c>
+      <c r="BW19" t="inlineStr">
+        <is>
+          <t>Qualifying (BANT), Setting Expectations, Close &amp; Confirmation, Objection Handling</t>
+        </is>
+      </c>
+      <c r="BX19" t="n">
+        <v>7</v>
+      </c>
+      <c r="BY19" t="inlineStr">
+        <is>
+          <t>Miles called Lions Roofing returning a missed callback and inquired whether the company handles small porch-roof repairs involving possible replacement of deteriorated wood/boarding beneath tile. Jackie explained that Lions Roofing does repairs and re-roofs, confirmed with a technician that they can address issues like fascia/plywood under tile, and noted a technician would need to come out to inspect and provide an estimate. Miles asked whether the technician would arrive with a ladder and in a marked Lions Roofing vehicle, which Jackie confirmed. Jackie offered availability for an appointment tomorrow (2026-03-14) in the morning or afternoon, but Miles chose not to schedule yet and said he would call back after consulting someone else.</t>
+        </is>
+      </c>
+      <c r="CA19" t="inlineStr">
+        <is>
+          <t>When can someone come by?, I do have availability tomorrow., What time?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/df6c19b0-5d39-457b-8053-4dd83f4407cf/4076546354.mp3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Jagger</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Roof inspection</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>I haven't received any information back from that as of yet.</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>follow_up_call</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Contact London today and tag him in the customer file to ensure he calls the customer back about the prior inspection and next steps</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>follow_up</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>customer_rep: How can I help you?
+customer_rep: Hello?
+home_owner: Yeah, this is a little bit of a weird question, but I called a roofer last week, and I think it was you, and I wanted to see if it was.
+home_owner: If I gave you my property address. Could you look up and see if you did an inspection last week?
+customer_rep: We did do an inspection on Tuesday, March 3rd.
+home_owner: Oh, you did? Okay, well, fantastic.
+home_owner: I'm glad that I got back to you.
+home_owner: I was wondering.
+home_owner: I haven't got.
+home_owner: I haven't received any information back from that as of yet.
+customer_rep: Okay.
+customer_rep: Yeah, it looks like London was the one who went out there.
+customer_rep: He's not in office today, but I will send him a text message and tag him in your file just so that he can either give you a call back and, like, get on the same page, or it might have just been.
+customer_rep: He didn't press send.
+home_owner: Okay.
+home_owner: Yeah, that's perfect.
+home_owner: Exactly what I was looking for.
+customer_rep: Sounds good.
+customer_rep: And then this is for Jagger, correct?
+home_owner: Yes.
+customer_rep: Okay, great.
+customer_rep: Yeah, I will go ahead and get in touch with London.
+home_owner: All right, sounds good.
+home_owner: Thank you.
+customer_rep: Have a good one.
+home_owner: All right, you too.
+customer_rep: Bye.
+home_owner: Bye.</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>scenario_test_9_e37ecbc8</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Customer rep to text London and tag him in the customer file so he follows up with the customer about the 2026-03-03 inspection results., Contact London today and tag him in the customer file to ensure he calls the customer back about the prior inspection and next steps</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="AG20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>in-person</t>
+        </is>
+      </c>
+      <c r="AM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>follow_up_inquiry</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>After the homeowner said they had not received any information from the inspection, the rep said they would text London and tag the file, but did not set a timeframe or explain what the customer should expect next (callback vs. email, and by when)., The call opened with a generic question and did not include the company name or a structured identification step; the rep also did not proactively verify contact information before ending the call.</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>Quickly located the prior inspection and identified the field rep responsible., Took ownership by committing to contact the inspector and tag the file., Confirmed the customer name before ending the call and closed politely.</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, </t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="AX20" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>Jagger (homeowner)</t>
+        </is>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>Customer (Jagger) is calling to confirm an inspection was done last week (Tuesday, March 3rd). They have not received any information/results yet. Rep noted inspector was London and will text/tag him to call customer back or send the info.</t>
+        </is>
+      </c>
+      <c r="BG20" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>Customer asked the company to look up whether they performed a roof inspection last week and requested the inspection information because they had not received anything back yet., Rep confirmed an inspection was completed on Tuesday, 2026-03-03, and that London was the inspector., Rep said London is not in the office on 2026-03-13 and will text him and tag him in the file so he can call the customer back; the account/file is for Jagger.</t>
+        </is>
+      </c>
+      <c r="BI20" t="inlineStr">
+        <is>
+          <t>London to call the customer to review the inspection findings and provide the missing follow-up information., Customer to await London’s callback for the inspection details.</t>
+        </is>
+      </c>
+      <c r="BJ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK20" t="inlineStr">
+        <is>
+          <t>Quickly located the prior inspection and identified the field rep responsible., Took ownership by committing to contact the inspector and tag the file., Confirmed the customer name before ending the call and closed politely.</t>
+        </is>
+      </c>
+      <c r="BM20" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO20" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP20" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="BQ20" t="inlineStr">
+        <is>
+          <t>Caller is following up on a recent roof inspection and has not yet received the inspection/estimate information, indicating an active pre-sale opportunity rather than post-contract production or service.</t>
+        </is>
+      </c>
+      <c r="BR20" t="inlineStr">
+        <is>
+          <t>follow-up on inspection/estimate, has not received information back yet, no contract/work scheduling/payment discussed</t>
+        </is>
+      </c>
+      <c r="BS20" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="BV20" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Confirm Project Details, Address Questions/Concerns, Close Professionally</t>
+        </is>
+      </c>
+      <c r="BW20" t="inlineStr">
+        <is>
+          <t>Set Expectations for Next Steps</t>
+        </is>
+      </c>
+      <c r="BX20" t="n">
+        <v>5</v>
+      </c>
+      <c r="BY20" t="inlineStr">
+        <is>
+          <t>The homeowner called to confirm whether this roofing company had performed an inspection at their property the prior week and to request the results, since they had not received any follow-up information. The customer service representative confirmed an inspection was completed on Tuesday, 2026-03-03, noted that London was the person who conducted it, and explained London was not in the office on the call date (2026-03-13). The representative committed to texting London and tagging him in the customer’s file so he can call the homeowner back and provide the inspection information, confirming the file is for Jagger before ending the call.</t>
+        </is>
+      </c>
+      <c r="CA20" t="inlineStr">
+        <is>
+          <t>I called a roofer last week, Could you look up and see if you did an inspection last week?, I haven't received any information back from that as of yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/6dd70da4-9d39-4496-871e-827af1429e29/4077402764.mp3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Diva</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Dora</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Roofing appointment/inspection (unspecified)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>not_booked</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Yes, hi. I just received a confirmation about a meeting, an appointment, rather, today between 11:30 and 12:30 here in Tucson. And that. I never coordinated that. And I've been talking directly to Rich, and we're trying to find a time that we could all meet. He didn't tell me that that time was available. Did something change? | Well, we. So we discussed that, you know, he's going to come out. He said something about tomorrow, but we're. We're leaving tomorrow.</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>confirm_appointment</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Contact Rich on 2026-03-13 to confirm the appointment status/time and ensure he does not go to the property until coordination is confirmed</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>confirmation</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>existing</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>customer_rep: Thank you for calling Arizona Roofers. My name is Diva. How can I help you?
+home_owner: Yes, hi. I just received a confirmation about a meeting, an appointment, rather, today between 11:30 and 12:30 here in Tucson. And that. I never coordinated that. And I've been talking directly to Rich, and we're trying to find a time that we could all meet. He didn't tell me that that time was available. Did something change?
+customer_rep: Okay, I'm not too sure. Let me take a look at the calendar. It could just be just like a tentative time.
+home_owner: What? I don't.
+customer_rep: Okay, yeah, I don't see that in your calendar. Okay, so I think maybe that was an accident. But, yeah, if you have Rich's information, you could just reach out to him.
+home_owner: Okay, great. I just didn't want to, you know.
+customer_rep: No, you're fine. Whatever he. Whatever he coordinated with you is what it. What it's going to be.
+home_owner: Okay, great. Thank you so much.
+customer_rep: Yeah, I'll also reach out to him and just double check that.
+home_owner: Yeah. Make sure that he doesn't go out there.
+customer_rep: I mean, what did you guys discuss?
+home_owner: Well, we. So we discussed that, you know, he's going to come out. He said something about tomorrow, but we're. We're leaving tomorrow. So I was going to connect him with my backup. And so he. And I said, rich, is that okay? Goes. Oh, yeah, absolutely. So I was going to, you know, connect him with the gentleman that kind of backs me up when I'm not here. And they were going to coordinate a time and a date, and that hasn't been established yet.
+customer_rep: Okay, interesting.
+home_owner: Yeah, this is Dora. Now, if. Yeah, this is so good. Now. Now, to be honest with you, if he were available today between 11:30 and 12:30, we could do it. I could do it. But Rich did. But he. What he said was tomorrow, which I'm not available until the end of the month, so. But if Rich is available during this time frame today, between 11:30 and 12:30, that would work.
+customer_rep: Okay, I'll go ahead and reach out to him and just see if he doesn't respond. You could try to reach out to him later on if you're. If he shows up. Or I guess we'll just play it by ear and see what goes on. I don't see a calendar event in here, so maybe it was a glitch in our system that you got that update. But if he is able to do it, I'll let him know that you're available today.
+home_owner: You know what? And I'll actually text him as well and say, hey, I got this confirmation for today, if you're available. We're available. But if not, I'm going to hook him up with my backup.
+customer_rep: Okay, perfect. Yep. That sounds great.
+home_owner: All right. Okay, awesome. Okay. Thanks so much.
+customer_rep: Of course. Have a good day.
+home_owner: You, too. Bye.
+customer_rep: Bye.</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>scenario_test_10_fcee5ce4</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Customer rep (Diva) to contact Rich to confirm whether he is scheduled to go to the Tucson property and to align on the correct appointment time., Contact Rich on 2026-03-13 to confirm the appointment status/time and ensure he does not go to the property until coordination is confirmed</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Tucson</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="AG21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>in-person</t>
+        </is>
+      </c>
+      <c r="AM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>qualified_but_unbooked</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>When the homeowner called about an appointment confirmation they 'never coordinated,' the rep said it was likely an accident/glitch and advised the customer to contact Rich, but did not verify key appointment details (what the system shows, correct date/time, address, who should be present) or provide a firm resolution/confirmation., The rep used vague/uncertain next steps instead of a clear plan, telling the customer to 'play it by ear' and suggesting they reach out later if Rich doesn't respond.</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>Provided a professional greeting with company name and rep name., Took ownership to follow up internally by offering to reach out to Rich and double-check.</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">, </t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>74%</t>
+        </is>
+      </c>
+      <c r="AX21" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="BB21" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BC21" t="inlineStr">
+        <is>
+          <t>Dora (homeowner), backup (gentleman that kind of backs me up when I'm not here)</t>
+        </is>
+      </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>Customer (Dora) received an appointment confirmation for today 11:30-12:30 in Tucson that she did not schedule. She has been coordinating directly with Rich; timing not established yet. She is available today 11:30-12:30 if Rich can come, otherwise she will connect Rich with her backup since she is leaving tomorrow and not available again until the end of the month. Rep to confirm with Rich to avoid an uncoordinated visit.</t>
+        </is>
+      </c>
+      <c r="BG21" t="b">
+        <v>1</v>
+      </c>
+      <c r="BH21" t="inlineStr">
+        <is>
+          <t>Customer received an appointment confirmation for 2026-03-13 (today) 11:30–12:30 in Tucson but says she never coordinated that time and was coordinating directly with Rich., Rep checked the company calendar and did not see the appointment, indicating it may have been an accidental/tentative booking or a system glitch., Customer said Rich mentioned coming out on 2026-03-14 (tomorrow) but she is leaving then; she can meet today 11:30–12:30 if Rich is available, otherwise she will connect Rich with her backup contact to coordinate a time/date.</t>
+        </is>
+      </c>
+      <c r="BI21" t="inlineStr">
+        <is>
+          <t>Diva will inform Rich that Dora is available on 2026-03-13 between 11:30 and 12:30 and confirm whether he can meet then., Dora will text Rich about the unexpected confirmation and, if needed, connect him with her backup contact to schedule a visit.</t>
+        </is>
+      </c>
+      <c r="BJ21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK21" t="inlineStr">
+        <is>
+          <t>Provided a professional greeting with company name and rep name., Took ownership to follow up internally by offering to reach out to Rich and double-check.</t>
+        </is>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="BO21" t="inlineStr">
+        <is>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="BP21" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="BQ21" t="inlineStr">
+        <is>
+          <t>Caller is clarifying and potentially scheduling an initial appointment/meeting with a salesperson (Rich) for a roof visit/inspection/estimate; no contract, production, payment, or warranty discussion.</t>
+        </is>
+      </c>
+      <c r="BR21" t="inlineStr">
+        <is>
+          <t>appointment/meeting coordination with sales rep, discussion of someone coming out to the property, pre-sale scheduling availability (today vs tomorrow/end of month)</t>
+        </is>
+      </c>
+      <c r="BS21" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="BT21" t="inlineStr">
+        <is>
+          <t>Tucson</t>
+        </is>
+      </c>
+      <c r="BV21" t="inlineStr">
+        <is>
+          <t>Greeting &amp; Identification, Answer Questions (if any), Close Professionally</t>
+        </is>
+      </c>
+      <c r="BW21" t="inlineStr">
+        <is>
+          <t>Confirm Appointment Details</t>
+        </is>
+      </c>
+      <c r="BX21" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY21" t="inlineStr">
+        <is>
+          <t>The homeowner (Dora) called after receiving an unexpected appointment confirmation for a roofing meeting in Tucson on 2026-03-13 between 11:30 and 12:30, stating she never coordinated that time and had been working directly with Rich to find a mutually available slot. The customer rep (Diva) checked the calendar, did not find the appointment, and suggested it may have been a system glitch or accidental tentative booking. Dora explained Rich had mentioned coming out on 2026-03-14, but she is leaving then and planned to connect Rich with her backup contact to coordinate a date/time that has not yet been set; however, if Rich is actually available during the 11:30–12:30 window today, she can meet. Diva said she would reach out to Rich to confirm and let him know Dora is available today, while Dora also planned to text Rich and, if needed, connect him with her backup so they can schedule.</t>
+        </is>
+      </c>
+      <c r="CA21" t="inlineStr">
+        <is>
+          <t>today between 11:30 and 12:30, tomorrow, we're leaving tomorrow, I'm not available until the end of the month</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3532,7 +6080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3763,6 +6311,206 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/bd24a254-fe4e-48ef-9c3e-3c3f3adfd68c/4082148782.mp3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>scenario_test_1_88148c4c</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/00273c23-da2c-4e1b-b49c-4ff85d4a766a/4082112377.mp3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>scenario_test_2_2e229983</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/c0183543-60e4-434f-a247-89ec9ef8e1e3/4081871096.mp3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>scenario_test_3_cc5d0fb9</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/eb359c0a-02e2-4e94-b018-b3585c8a4024/4081765241.mp3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>scenario_test_4_334fff68</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/4da88a74-f129-481d-92d4-626c5a728835/4081742162.mp3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>scenario_test_5_8b5c1e22</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/c6c4fff3-72d5-42d5-9cb4-16b8272e3d3b/4079556188.mp3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>scenario_test_6_c383236d</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/ddccb9c0-fce8-4eb5-81bd-5e738cb95979/4078581674.mp3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>scenario_test_7_b228486b</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/add722b1-c29f-4615-b389-4d29773d5958/st_309419607.mp3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>scenario_test_8_a99fa915</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/df6c19b0-5d39-457b-8053-4dd83f4407cf/4076546354.mp3</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>scenario_test_9_e37ecbc8</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://ottoaudio.s3.ap-southeast-2.amazonaws.com/recordings/6dd70da4-9d39-4496-871e-827af1429e29/4077402764.mp3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>scenario_test_10_fcee5ce4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>